<commit_message>
data(gold-gears): G08-P3-B5 author complete workbooks
</commit_message>
<xml_diff>
--- a/config/gold-and-gears-generated/templates/GoldAndGears.xlsx
+++ b/config/gold-and-gears-generated/templates/GoldAndGears.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2614" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2595" uniqueCount="241">
   <si>
     <t>@table</t>
   </si>
@@ -320,7 +320,7 @@
     <t>GoldGearsMapNode</t>
   </si>
   <si>
-    <t>089cb018aeb0516d</t>
+    <t>870db2e516229954</t>
   </si>
   <si>
     <t>column_id</t>
@@ -434,82 +434,67 @@
     <t>GoldGearsBeacon</t>
   </si>
   <si>
-    <t>8c8958e62bb93ea6</t>
-  </si>
-  <si>
-    <t>modifier_name</t>
-  </si>
-  <si>
-    <t>modifier_name_hash</t>
+    <t>44349503020bfd79</t>
+  </si>
+  <si>
+    <t>GoldGearsBossChoice</t>
+  </si>
+  <si>
+    <t>0cf26273bf658cd1</t>
+  </si>
+  <si>
+    <t>display_level</t>
+  </si>
+  <si>
+    <t>weakness_elements</t>
+  </si>
+  <si>
+    <t>monster_template_id</t>
+  </si>
+  <si>
+    <t>GoldGearsCognitionRange</t>
+  </si>
+  <si>
+    <t>acb8e695b392f044</t>
+  </si>
+  <si>
+    <t>area_stable_key</t>
+  </si>
+  <si>
+    <t>minimum_cognition</t>
+  </si>
+  <si>
+    <t>maximum_cognition</t>
+  </si>
+  <si>
+    <t>bounds_inclusive</t>
+  </si>
+  <si>
+    <t>global_minimum_cognition</t>
+  </si>
+  <si>
+    <t>global_maximum_cognition</t>
+  </si>
+  <si>
+    <t>lifecycle_json</t>
+  </si>
+  <si>
+    <t>GoldGearsModeConstant</t>
+  </si>
+  <si>
+    <t>1b426f4bd4cebb39</t>
+  </si>
+  <si>
+    <t>mechanical_role</t>
+  </si>
+  <si>
+    <t>value_kind</t>
+  </si>
+  <si>
+    <t>values</t>
   </si>
   <si>
     <t>length=1..200</t>
-  </si>
-  <si>
-    <t>GoldGearsBossChoice</t>
-  </si>
-  <si>
-    <t>ea66d6ebac4f3ce3</t>
-  </si>
-  <si>
-    <t>area_id</t>
-  </si>
-  <si>
-    <t>monster_id</t>
-  </si>
-  <si>
-    <t>monster_template_id</t>
-  </si>
-  <si>
-    <t>enemy_variant_stable_key</t>
-  </si>
-  <si>
-    <t>display_order</t>
-  </si>
-  <si>
-    <t>ref&lt;GoldGearsArea.id&gt;</t>
-  </si>
-  <si>
-    <t>GoldGearsCognitionRange</t>
-  </si>
-  <si>
-    <t>acb8e695b392f044</t>
-  </si>
-  <si>
-    <t>area_stable_key</t>
-  </si>
-  <si>
-    <t>minimum_cognition</t>
-  </si>
-  <si>
-    <t>maximum_cognition</t>
-  </si>
-  <si>
-    <t>bounds_inclusive</t>
-  </si>
-  <si>
-    <t>global_minimum_cognition</t>
-  </si>
-  <si>
-    <t>global_maximum_cognition</t>
-  </si>
-  <si>
-    <t>lifecycle_json</t>
-  </si>
-  <si>
-    <t>GoldGearsModeConstant</t>
-  </si>
-  <si>
-    <t>1b426f4bd4cebb39</t>
-  </si>
-  <si>
-    <t>mechanical_role</t>
-  </si>
-  <si>
-    <t>value_kind</t>
-  </si>
-  <si>
-    <t>values</t>
   </si>
   <si>
     <t>parser=split;separator=|;length=1..256</t>
@@ -2686,7 +2671,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2699,11 +2684,9 @@
     <col min="12" max="12" width="30.7109375" style="5" customWidth="1"/>
     <col min="13" max="14" width="22.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="12.7109375" style="5" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="18.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2735,7 +2718,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="24" customHeight="1">
+    <row r="2" spans="1:15" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -2781,14 +2764,8 @@
       <c r="O2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="P2" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17">
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" s="4" t="s">
         <v>30</v>
       </c>
@@ -2834,14 +2811,8 @@
       <c r="O3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="P3" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17">
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" s="4" t="s">
         <v>31</v>
       </c>
@@ -2887,14 +2858,8 @@
       <c r="O4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="P4" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17">
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" s="4" t="s">
         <v>40</v>
       </c>
@@ -2940,14 +2905,8 @@
       <c r="O5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q5" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17">
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" s="4" t="s">
         <v>41</v>
       </c>
@@ -2987,14 +2946,8 @@
       <c r="O6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="P6" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="Q6" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" ht="42" customHeight="1">
+    </row>
+    <row r="7" spans="1:15" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>49</v>
       </c>
@@ -3012,8 +2965,6 @@
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
       <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -3037,7 +2988,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -3050,19 +3001,17 @@
     <col min="12" max="12" width="30.7109375" style="5" customWidth="1"/>
     <col min="13" max="14" width="22.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="12.7109375" style="5" customWidth="1"/>
-    <col min="16" max="16" width="21.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="17.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="19.7109375" style="5" customWidth="1"/>
-    <col min="19" max="19" width="24.7109375" style="5" customWidth="1"/>
-    <col min="20" max="20" width="13.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3086,10 +3035,10 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" ht="24" customHeight="1">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -3136,22 +3085,16 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
       <c r="A3" s="4" t="s">
         <v>30</v>
       </c>
@@ -3198,22 +3141,16 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
       <c r="A4" s="4" t="s">
         <v>31</v>
       </c>
@@ -3260,22 +3197,16 @@
         <v>33</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>143</v>
+        <v>32</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="S4" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="T4" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20">
+    </row>
+    <row r="5" spans="1:18">
       <c r="A5" s="4" t="s">
         <v>40</v>
       </c>
@@ -3330,14 +3261,8 @@
       <c r="R5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="S5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="T5" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20">
+    </row>
+    <row r="6" spans="1:18">
       <c r="A6" s="4" t="s">
         <v>41</v>
       </c>
@@ -3377,21 +3302,17 @@
       <c r="O6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="P6" s="5"/>
+      <c r="P6" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="Q6" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="S6" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="T6" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" ht="42" customHeight="1">
+    </row>
+    <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>49</v>
       </c>
@@ -3412,8 +3333,6 @@
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
-      <c r="T7" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="5">
@@ -3430,9 +3349,9 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="GoldGearsEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 0 to 100." promptTitle="Integer range" prompt="Enter an integer from 0 to 100." sqref="T8:T1007">
-      <formula1>0</formula1>
-      <formula2>100</formula2>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 200." promptTitle="Integer range" prompt="Enter an integer from 1 to 200." sqref="P8:P1007">
+      <formula1>1</formula1>
+      <formula2>200</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3466,7 +3385,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3490,7 +3409,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="24" customHeight="1">
@@ -3540,25 +3459,25 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="V2" s="3" t="s">
         <v>146</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -3608,25 +3527,25 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="V3" s="5" t="s">
         <v>146</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -3898,7 +3817,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3922,7 +3841,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -3972,13 +3891,13 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -4028,13 +3947,13 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -4187,7 +4106,7 @@
         <v>48</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="P6" s="5" t="s">
         <v>45</v>
@@ -4196,7 +4115,7 @@
         <v>44</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
@@ -4265,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4289,7 +4208,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -4339,13 +4258,13 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -4395,13 +4314,13 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -4557,7 +4476,7 @@
         <v>61</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>61</v>
@@ -4650,7 +4569,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4674,7 +4593,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:33" ht="24" customHeight="1">
@@ -4724,58 +4643,58 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="Q2" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="W2" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="X2" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="S2" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="T2" s="3" t="s">
+      <c r="Y2" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>170</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="W2" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="X2" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="Y2" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="Z2" s="3" t="s">
-        <v>175</v>
       </c>
       <c r="AA2" s="3" t="s">
         <v>26</v>
       </c>
       <c r="AB2" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC2" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="AD2" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="AE2" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="AF2" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="AG2" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="AC2" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="AD2" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="AE2" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AF2" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="AG2" s="3" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:33">
@@ -4825,58 +4744,58 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="Q3" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="W3" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="X3" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="S3" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="T3" s="5" t="s">
+      <c r="Y3" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="U3" s="5" t="s">
+      <c r="Z3" s="5" t="s">
         <v>170</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="Y3" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>175</v>
       </c>
       <c r="AA3" s="5" t="s">
         <v>26</v>
       </c>
       <c r="AB3" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC3" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="AD3" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="AE3" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="AF3" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="AG3" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="AC3" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="AD3" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="AE3" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="AF3" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="AG3" s="5" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:33">
@@ -4929,7 +4848,7 @@
         <v>32</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>33</v>
@@ -5122,7 +5041,7 @@
         <v>61</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="Q6" s="5"/>
       <c r="R6" s="5" t="s">
@@ -5155,10 +5074,10 @@
         <v>61</v>
       </c>
       <c r="AC6" s="5" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="AD6" s="5" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="AE6" s="5" t="s">
         <v>48</v>
@@ -5266,7 +5185,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5290,7 +5209,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="24" customHeight="1">
@@ -5340,34 +5259,34 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="V2" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="W2" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="X2" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="Y2" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="W2" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="X2" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="Y2" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -5417,34 +5336,34 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="V3" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="W3" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="X3" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="T3" s="5" t="s">
+      <c r="Y3" s="5" t="s">
         <v>190</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="Y3" s="5" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -5494,7 +5413,7 @@
         <v>33</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>33</v>
@@ -6219,7 +6138,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6243,7 +6162,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="24" customHeight="1">
@@ -6293,28 +6212,28 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="V2" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="W2" s="3" t="s">
         <v>201</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="W2" s="3" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -6364,28 +6283,28 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="V3" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="W3" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -6453,7 +6372,7 @@
         <v>32</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="W4" s="5" t="s">
         <v>32</v>
@@ -6571,26 +6490,26 @@
         <v>61</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>61</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="T6" s="5" t="s">
         <v>61</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="V6" s="5"/>
       <c r="W6" s="5" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="42" customHeight="1">
@@ -6691,7 +6610,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6715,7 +6634,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:36" ht="24" customHeight="1">
@@ -6765,67 +6684,67 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="Q2" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="Y2" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="AA2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="T2" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="W2" s="3" t="s">
+      <c r="AB2" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="AC2" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="Y2" s="3" t="s">
+      <c r="AD2" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="Z2" s="3" t="s">
+      <c r="AE2" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="AA2" s="3" t="s">
+      <c r="AF2" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="AB2" s="3" t="s">
+      <c r="AG2" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AH2" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="AD2" s="3" t="s">
+      <c r="AI2" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="AE2" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="AF2" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="AG2" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="AH2" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="AI2" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="AJ2" s="3" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:36">
@@ -6875,67 +6794,67 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="Q3" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="Y3" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="Z3" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="AA3" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="T3" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="W3" s="5" t="s">
+      <c r="AB3" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="X3" s="5" t="s">
+      <c r="AC3" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="Y3" s="5" t="s">
+      <c r="AD3" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="Z3" s="5" t="s">
+      <c r="AE3" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="AA3" s="5" t="s">
+      <c r="AF3" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="AB3" s="5" t="s">
+      <c r="AG3" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="AC3" s="5" t="s">
+      <c r="AH3" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="AD3" s="5" t="s">
+      <c r="AI3" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="AE3" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="AF3" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="AG3" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="AH3" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="AI3" s="5" t="s">
-        <v>227</v>
-      </c>
       <c r="AJ3" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:36">
@@ -7199,13 +7118,13 @@
         <v>61</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>61</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="S6" s="5" t="s">
         <v>90</v>
@@ -7363,7 +7282,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7387,7 +7306,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -7437,19 +7356,19 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -7499,19 +7418,19 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -7679,7 +7598,7 @@
         <v>61</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>61</v>
@@ -7689,7 +7608,7 @@
       </c>
       <c r="S6" s="5"/>
       <c r="T6" s="5" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="42" customHeight="1">
@@ -7776,7 +7695,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7800,7 +7719,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="24" customHeight="1">
@@ -7850,40 +7769,40 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="V2" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y2" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="AA2" s="3" t="s">
         <v>239</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="W2" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="X2" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="Y2" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="Z2" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:27">
@@ -7933,40 +7852,40 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="V3" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y3" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="Z3" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="AA3" s="5" t="s">
         <v>239</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="Y3" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="AA3" s="5" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:27">
@@ -8016,7 +7935,7 @@
         <v>33</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>33</v>
@@ -9759,7 +9678,8 @@
     <col min="15" max="15" width="12.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="27.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="26.7109375" style="5" customWidth="1"/>
-    <col min="18" max="20" width="12.7109375" style="5" customWidth="1"/>
+    <col min="18" max="19" width="12.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="22.7109375" style="5" customWidth="1"/>
     <col min="21" max="21" width="17.7109375" style="5" customWidth="1"/>
     <col min="22" max="23" width="12.7109375" style="5" customWidth="1"/>
   </cols>
@@ -9997,7 +9917,7 @@
         <v>32</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="U4" s="5" t="s">
         <v>33</v>
@@ -10129,7 +10049,7 @@
         <v>91</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>44</v>

</xml_diff>